<commit_message>
Add more images/updated robot design to readme
</commit_message>
<xml_diff>
--- a/CAD/Inventor/parameters.xlsx
+++ b/CAD/Inventor/parameters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\satom\Desktop\Robot\CAD\Inventor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C210662A-4F41-41B6-BF7D-0CC7009CABE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E197D568-6794-4528-8736-36AC5676562E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="7530" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="59430" yWindow="9480" windowWidth="21600" windowHeight="10920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -395,6 +395,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <cols>
+    <col min="1" max="1" width="21.7890625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">

</xml_diff>